<commit_message>
Refactor draw_name function for improved layout and font sizing in nameplate generation
</commit_message>
<xml_diff>
--- a/名簿・領収書.xlsx
+++ b/名簿・領収書.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\matu\work\ToDo\support-ac\python\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\matu\work\ToDo\support-ac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A259773-CA37-43BD-95BD-82E828A728ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B68C67-88C1-48BE-A927-F887C7C99BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="-3705" windowWidth="29010" windowHeight="32505" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="参加費" sheetId="1" r:id="rId1"/>
@@ -59,12 +59,6 @@
     <t>一般</t>
   </si>
   <si>
-    <t>参加者2</t>
-  </si>
-  <si>
-    <t>参加者3</t>
-  </si>
-  <si>
     <t>参加者4</t>
   </si>
   <si>
@@ -218,20 +212,40 @@
     <phoneticPr fontId="5"/>
   </si>
   <si>
-    <t>長～～～～～～～～～～～～～～～～～～～～～い所属</t>
-  </si>
-  <si>
-    <t>長～～～～～～～～～～～～～～～～い所属</t>
-  </si>
-  <si>
-    <t>長～～～～～～い所属</t>
-  </si>
-  <si>
     <t>所属</t>
     <phoneticPr fontId="5"/>
   </si>
   <si>
-    <t>長～～～～～～～～～～～い所属</t>
+    <t>長～２５文字～～～～～～～～～～～～～～～～い所属</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>長～２０文字～～～～～～～～～～～い所属</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>長～１５文字～～～～～～い所属</t>
+    <rPh sb="4" eb="6">
+      <t>モジ</t>
+    </rPh>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>長～１０文字～い所属</t>
+    <rPh sb="4" eb="6">
+      <t>モジ</t>
+    </rPh>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>参加者3_１０文字</t>
+    <rPh sb="7" eb="9">
+      <t>モジ</t>
+    </rPh>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>sankasya_long_name</t>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -242,7 +256,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="#,##0_);[Red]\(#,##0\)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -674,7 +688,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AMD26"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="14.77734375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.44140625" style="1" customWidth="1"/>
@@ -686,30 +700,30 @@
     <col min="1019" max="1020" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="14.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -733,12 +747,12 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
@@ -757,12 +771,12 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
@@ -781,12 +795,12 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
@@ -805,9 +819,9 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>57</v>
@@ -829,12 +843,12 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>5</v>
@@ -853,12 +867,12 @@
         <v>17000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>5</v>
@@ -877,12 +891,12 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>5</v>
@@ -901,12 +915,12 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>5</v>
@@ -925,12 +939,12 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>5</v>
@@ -949,15 +963,15 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="D12" s="2">
         <v>2000</v>
@@ -973,15 +987,15 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D13" s="2">
         <v>2000</v>
@@ -997,15 +1011,15 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D14" s="2">
         <v>0</v>
@@ -1021,15 +1035,15 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D15" s="2">
         <v>2000</v>
@@ -1045,15 +1059,15 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2">
         <v>2000</v>
@@ -1069,15 +1083,15 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D17" s="2">
         <v>3000</v>
@@ -1093,15 +1107,15 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D18" s="2">
         <v>3000</v>
@@ -1117,15 +1131,15 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D19" s="2">
         <v>3000</v>
@@ -1141,15 +1155,15 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D20" s="2">
         <v>3000</v>
@@ -1165,15 +1179,15 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D21" s="2">
         <v>3000</v>
@@ -1189,63 +1203,63 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7">
       <c r="A22" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="D22" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E22" s="2">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2">
+        <v>5000</v>
+      </c>
+      <c r="G22" s="2">
+        <f t="shared" si="0"/>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="2">
-        <v>5000</v>
-      </c>
-      <c r="E22" s="2">
-        <v>0</v>
-      </c>
-      <c r="F22" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G22" s="2">
-        <f t="shared" si="0"/>
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
+      <c r="C23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2">
+        <v>5000</v>
+      </c>
+      <c r="G23" s="2">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="2">
-        <v>0</v>
-      </c>
-      <c r="E23" s="2">
-        <v>0</v>
-      </c>
-      <c r="F23" s="2">
-        <v>5000</v>
-      </c>
-      <c r="G23" s="2">
-        <f t="shared" si="0"/>
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="C24" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D24" s="2">
         <v>5000</v>
@@ -1261,15 +1275,15 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7">
       <c r="A25" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D25" s="2">
         <v>6000</v>
@@ -1285,15 +1299,15 @@
         <v>11000</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D26" s="2">
         <v>6000</v>

</xml_diff>

<commit_message>
Update Excel file with new data and formatting changes
</commit_message>
<xml_diff>
--- a/名簿・領収書.xlsx
+++ b/名簿・領収書.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\matu\work\ToDo\support-ac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B68C67-88C1-48BE-A927-F887C7C99BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E7D847-1CCF-4A90-991B-2F01E5062AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3936" yWindow="3936" windowWidth="11532" windowHeight="7620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="参加費" sheetId="1" r:id="rId1"/>
@@ -700,7 +700,7 @@
     <col min="1019" max="1020" width="9.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>